<commit_message>
feat: Sprint 1 terminé - fiche produit dynamique
</commit_message>
<xml_diff>
--- a/docs/Box GardeMeuble.xlsx
+++ b/docs/Box GardeMeuble.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acboi\Documents\Projets\vente-meubles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acboi\Documents\Projets\vente-meubles\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB1C177F-0731-4A24-A740-FB0BEBB23C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1602A8-23C2-4DA8-9974-058790104991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FD343005-4382-4935-A274-266D1E9B84BE}"/>
   </bookViews>
@@ -939,10 +939,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
FEAT-017b : Corrections des écrans - Responsive
</commit_message>
<xml_diff>
--- a/docs/Box GardeMeuble.xlsx
+++ b/docs/Box GardeMeuble.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acboi\Documents\Projets\vente-meubles\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EFB301-8C88-4D8B-BE21-D75E2B492504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0449EA4D-755D-4D8F-B17E-27AE53AD8FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FD343005-4382-4935-A274-266D1E9B84BE}"/>
   </bookViews>
@@ -259,35 +259,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Meuble TV 155 cm TOMY coloris chêne et noir </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Style industriel et élégance moderne
-Le meuble TV 155 cm TOMY coloris chêne et noir de  s'intègre parfaitement dans un intérieur au style industriel. Son design bicolore, associant le chêne jackson et le noir, apporte une touche de modernité et de sophistication à votre salon. Ce meuble est idéal pour créer une ambiance chaleureuse et accueillante, tout en offrant un espace de rangement pratique pour votre équipement multimédia. Avec ses lignes épurées et sa finition en papier décor, il se marie aisément avec divers styles de décoration, du contemporain au vintage.
-Fabrication française et fonctionnalité optimale
-Fabriqué en France, le meuble TV TOMY garantit une qualité de fabrication irréprochable. Conçu à partir de panneaux de particules, il offre une robustesse et une durabilité appréciables. Ce meuble est doté d'une porte coulissante, permettant un accès facile à vos appareils électroniques tout en les protégeant de la poussière. Une tablette de rangement supplémentaire est intégrée, idéale pour organiser vos accessoires multimédia. Le passe-câbles intégré assure une gestion discrète et ordonnée des fils, contribuant à un espace de vie harmonieux et bien rangé.
-Dimensions généreuses et choix de coloris
-Avec une longueur de 155 cm, une largeur de 40 cm et une hauteur de 43 cm, le meuble TV TOMY offre un espace suffisant pour accueillir une grande télévision ainsi que d'autres équipements audiovisuels. Son poids total de 24 kg témoigne de sa solidité et de sa stabilité. Disponible en deux coloris, chêne jackson/noir et chêne jackson/blanc, ce meuble s'adapte à vos préférences esthétiques et à l'agencement de votre pièce. Le choix des teintes permet de personnaliser votre intérieur tout en maintenant une cohérence visuelle avec le reste de votre mobilier.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Ensemble table rectangulaire 4 chaises TONY</t>
     </r>
     <r>
@@ -375,34 +346,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Un style industriel moderne</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Le lit adulte WATSON de CONFORAMA s'illustre par son style industriel, idéal pour ceux qui souhaitent insuffler une ambiance moderne et épurée à leur chambre. Avec sa finition en papier décor et ses teintes chêne kronberg et waterford, ce lit apporte une légère touche industrielle, tout en restant chaleureux. Sa tête de lit se distingue par un travail sur les contrastes, offrant ainsi un design unique qui s'intègre parfaitement dans un intérieur contemporain.
-Fabrication française et matériaux de qualité
-Fabriqué en France, le lit WATSON garantit une qualité et un savoir-faire exceptionnels. Sa structure est conçue en panneau de particules de 15 et 18 mm, assurant robustesse et durabilité. Bien que vendu sans sommier ni matelas, ce lit offre une base solide pour accueillir le couchage de votre choix. La fabrication française est un gage de qualité, et ce modèle s'inscrit parfaitement dans cette tradition d'excellence.
-Dimensions optimales et coloris bois clair
-Le lit WATSON propose des dimensions de couchage de 140x190 cm, adaptées aux besoins d'un lit simple. Avec une longueur de 194,7 cm, une largeur de 148,3 cm et une hauteur de 71,7 cm, il s'intègre facilement dans la plupart des espaces. Son coloris bois clair apporte une touche de luminosité et de douceur à votre chambre, créant une atmosphère apaisante. Disponible également en teinte blanche, ce lit s'adapte à vos préférences et à votre décoration intérieure.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Chevet WATSON : Design industriel et fabrication française</t>
     </r>
     <r>
@@ -432,40 +375,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Matelas 140x190 cm 8 HEURES FUTE : Confort et soutien optimal fabriqué en France</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Confort sur mesure pour des nuits paisibles
-Le matelas 140x190 cm 8 HEURES FUTE est un choix idéal pour ceux qui recherchent un confort équilibré et un soutien medium. Grâce à sa technologie de ressorts ensachés, ce matelas offre une indépendance de couchage remarquable, permettant de ne pas ressentir les mouvements de son partenaire. Fabriqué en France, il répond aux besoins des couples ou des personnes seules souhaitant un matelas deux places qui s'adapte parfaitement à leur morphologie. Son accueil ferme et son épaisseur de 21 cm garantissent un sommeil réparateur, quelle que soit la saison.
-Technologie avancée et fabrication française
-Ce matelas 8 HEURES FUTE se distingue par sa suspension de 480 ressorts ensachés, qui assure une excellente circulation de l'air et un soutien durable. Le tissu stretch 100 % polyester optimise la ventilation, évacuant l'humidité pour un confort optimal. Avec ses deux faces de couchage, il s'adapte aux variations saisonnières, offrant une face été avec un garnissage fin et respirant, et une face hiver plus enveloppante. Sa fabrication en France est un gage de qualité, garantissant un produit conforme aux normes les plus exigeantes.
-Un matelas pour tous les dormeurs
-Le matelas 140x190 cm 8 HEURES FUTE est conçu pour s'adresser à un large public. Que vous soyez un couple ou une personne seule, ce matelas deux places s'intègre parfaitement dans votre chambre. Son soutien medium et son accueil ferme conviennent à ceux qui recherchent un équilibre entre fermeté et moelleux. Avec un poids de 32 kg, il est à la fois robuste et facile à manipuler. Ce matelas est idéal pour ceux qui souhaitent investir dans un produit de qualité, fabriqué en France, qui assure des nuits paisibles et confortables.
-8 HEURES : LE BONHEUR ÇA COMMENCE PAR DE BELLES NUITS
-Parce qu’on vous connaît bien et que l’on a envie que vos nuits soient encore plus belles, nous avons créé 8 HEURES, une marque exclusive, inspirée par vous, qui allie confort, fiabilité, et accessibilité.
-Découvrez le bonheur de vous détendre avec des produits de qualité dans tout l’univers de la nuit, à des prix très accessibles.
-Parce que le bonheur de bien dormir n’a pas de prix, ou bien un tout petit, nos gammes s’adapteront parfaitement à vos besoins, vos envies et vos possibilités. Quel que soit votre choix, optez pour le confort maximum avec nos matelas, sommiers, couettes, oreillers… bien pensés pour chaque type de sommeil et chaque type de dormeur.
-Parce que tout le monde a le droit à un meilleur sommeil. Alors, pour mieux dormir toutes les nuits, reposez-vous sur notre marque exclusive : 8 HEURES.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>Cadre à lattes fixe 140x190 cm NIGHTITUDE C34 F07 : confort et soutien optimal</t>
     </r>
     <r>
@@ -483,35 +392,6 @@
 Fabriqué en France, ce sommier tapissier se distingue par ses caractéristiques techniques avancées. Avec une longueur de 190 cm, une largeur de 140 cm et une épaisseur de 5 cm, il s'intègre parfaitement dans les chambres de taille moyenne. Le choix de matériaux de qualité comme le métal pour la structure et les lattes multiplis pour la suspension assure une durabilité exceptionnelle. De plus, son coloris gris s'harmonise facilement avec tout type de décor. L'origine française de ce produit est un gage de qualité et de savoir-faire, renforçant ainsi sa position sur le marché.
 Un sommier adapté à tous les besoins
 Ce sommier pour 2 personnes est conçu pour s'adapter à tous les types de matelas, offrant ainsi une grande flexibilité d'utilisation. Il est idéal pour les couples ou les personnes seules qui préfèrent un espace de couchage plus spacieux. Avec un poids total de 16 kg, il est facile à manipuler lors de l'installation. Ce sommier en bois est parfait pour ceux qui recherchent un produit fiable et esthétique, tout en bénéficiant d'un excellent rapport qualité/prix. Sa fabrication en France et ses caractéristiques techniques en font un choix de prédilection pour ceux qui souhaitent investir dans un produit durable et performant.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Armoire WATSON : Élégance et fonctionnalité made in France</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Design naturel et moderne
-L'armoire 3 portes battantes WATSON se distingue par son design moderne et épuré, alliant le coloris Chêne Kronberg et Waterford. Ce meuble au style naturel s'intègre parfaitement dans tout type d'intérieur, qu'il soit contemporain ou plus classique. Grâce à son miroir intégré, elle agrandit visuellement l'espace et apporte une luminosité supplémentaire à votre pièce. Fabriquée en France, cette armoire allie esthétisme et qualité, répondant ainsi aux attentes des consommateurs soucieux de l'origine de fabrication de leurs meubles.
-Fonctionnalités et caractéristiques techniques
-Dotée de 3 portes battantes, l'armoire WATSON offre un aménagement intérieur astucieux avec deux tiers dédiés à la penderie et un tiers en lingère. Les étagères modulables permettent de ranger efficacement vos vêtements pliés. La structure en panneau de particules assure une robustesse et une durabilité optimales. Les poignées en plastique ajoutent une touche de modernité tout en étant pratiques. Avec une largeur de 133,5 cm, une hauteur de 191,5 cm et une profondeur de 51,4 cm, cette armoire est conçue pour optimiser l'espace de rangement tout en s'adaptant à des pièces de tailles variées. Sa finition en papier décor lui confère une allure soignée et élégante.
-Un meuble pour tous les foyers
-L'armoire WATSON est idéale pour ceux qui recherchent un meuble à la fois fonctionnel et esthétique. Elle s'adresse aux familles souhaitant organiser efficacement leur espace de rangement, ainsi qu'aux personnes vivant en appartement qui désirent maximiser leur espace. Grâce à sa fabrication française, elle séduit les consommateurs attachés à la qualité et à l'origine de leurs produits. Que ce soit pour une chambre d'adulte ou une chambre d'adolescent, cette armoire s'adapte à tous les besoins et styles de vie. Disponible également en coloris blanc, elle offre une flexibilité supplémentaire pour s'harmoniser avec votre décoration intérieure.</t>
     </r>
   </si>
   <si>
@@ -618,6 +498,158 @@
   </si>
   <si>
     <t>noir d'encre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">surface PU résistante à l'usure </t>
+  </si>
+  <si>
+    <t>teintes chêne kronberg et waterford</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> tissu stretch 100 % polyester</t>
+  </si>
+  <si>
+    <t>Blanc</t>
+  </si>
+  <si>
+    <t>métal</t>
+  </si>
+  <si>
+    <t>noir avec un plateau et des crochets en bois</t>
+  </si>
+  <si>
+    <t>coloris naturel et noir</t>
+  </si>
+  <si>
+    <t>Bois et Métal</t>
+  </si>
+  <si>
+    <t>Table séjour +4 chaises</t>
+  </si>
+  <si>
+    <t>Lot de 2 Chevets</t>
+  </si>
+  <si>
+    <t>Armoire 3 portes battante</t>
+  </si>
+  <si>
+    <t>Lot de 2 meubles WC</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Armoire WATSON : Élégance et fonctionnalité made in France</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Design naturel et moderne
+L'armoire 3 portes battantes WATSON se distingue par son design moderne et épuré, alliant le coloris Chêne Kronberg et Waterford. Ce meuble au style naturel s'intègre parfaitement dans tout type d'intérieur, qu'il soit contemporain ou plus classique. Grâce à son miroir intégré, elle agrandit visuellement l'espace et apporte une luminosité supplémentaire à votre pièce. Fabriquée en France, cette armoire allie esthétisme et qualité, répondant ainsi aux attentes des consommateurs soucieux de l'origine de fabrication de leurs meubles.
+Fonctionnalités et caractéristiques techniques
+Dotée de 3 portes battantes, l'armoire WATSON offre un aménagement intérieur astucieux avec deux tiers dédiés à la penderie et un tiers en lingère. Les étagères modulables permettent de ranger efficacement vos vêtements pliés. La structure en panneau de particules assure une robustesse et une durabilité optimales. Les poignées en plastique ajoutent une touche de modernité tout en étant pratiques. Avec une largeur de 133,5 cm, une hauteur de 191,5 cm et une profondeur de 51,4 cm, cette armoire est conçue pour optimiser l'espace de rangement tout en s'adaptant à des pièces de tailles variées. Sa finition en papier décor lui confère une allure soignée et élégante.
+Un meuble pour tous les foyers
+L'armoire WATSON est idéale pour ceux qui recherchent un meuble à la fois fonctionnel et esthétique. Elle s'adresse aux familles souhaitant organiser efficacement leur espace de rangement, ainsi qu'aux personnes vivant en appartement qui désirent maximiser leur espace. Grâce à sa fabrication française, elle séduit les consommateurs attachés à la qualité et à l'origine de leurs produits. Que ce soit pour une chambre d'adulte ou une chambre d'adolescent, cette armoire s'adapte à tous les besoins et styles de vie. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Meuble TV 155 cm TOMY coloris chêne et noir </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Style industriel et élégance moderne
+Le meuble TV 155 cm TOMY coloris chêne et noir de  s'intègre parfaitement dans un intérieur au style industriel. Son design bicolore, associant le chêne jackson et le noir, apporte une touche de modernité et de sophistication à votre salon. Ce meuble est idéal pour créer une ambiance chaleureuse et accueillante, tout en offrant un espace de rangement pratique pour votre équipement multimédia. Avec ses lignes épurées et sa finition en papier décor, il se marie aisément avec divers styles de décoration, du contemporain au vintage.
+Fabrication française et fonctionnalité optimale
+Fabriqué en France, le meuble TV TOMY garantit une qualité de fabrication irréprochable. Conçu à partir de panneaux de particules, il offre une robustesse et une durabilité appréciables. Ce meuble est doté d'une porte coulissante, permettant un accès facile à vos appareils électroniques tout en les protégeant de la poussière. Une tablette de rangement supplémentaire est intégrée, idéale pour organiser vos accessoires multimédia. Le passe-câbles intégré assure une gestion discrète et ordonnée des fils, contribuant à un espace de vie harmonieux et bien rangé.
+Dimensions généreuses et choix de coloris
+Avec une longueur de 155 cm, une largeur de 40 cm et une hauteur de 43 cm, le meuble TV TOMY offre un espace suffisant pour accueillir une grande télévision ainsi que d'autres équipements audiovisuels. Son poids total de 24 kg témoigne de sa solidité et de sa stabilité. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Un style industriel moderne</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Le lit adulte WATSON de CONFORAMA s'illustre par son style industriel, idéal pour ceux qui souhaitent insuffler une ambiance moderne et épurée à leur chambre. Avec sa finition en papier décor et ses teintes chêne kronberg et waterford, ce lit apporte une légère touche industrielle, tout en restant chaleureux. Sa tête de lit se distingue par un travail sur les contrastes, offrant ainsi un design unique qui s'intègre parfaitement dans un intérieur contemporain.
+Fabrication française et matériaux de qualité
+Fabriqué en France, le lit WATSON garantit une qualité et un savoir-faire exceptionnels. Sa structure est conçue en panneau de particules de 15 et 18 mm, assurant robustesse et durabilité. Bien que vendu sans sommier ni matelas, ce lit offre une base solide pour accueillir le couchage de votre choix. La fabrication française est un gage de qualité, et ce modèle s'inscrit parfaitement dans cette tradition d'excellence.
+Dimensions optimales et coloris bois clair
+Le lit WATSON propose des dimensions de couchage de 140x190 cm, adaptées aux besoins d'un lit simple. Avec une longueur de 194,7 cm, une largeur de 148,3 cm et une hauteur de 71,7 cm, il s'intègre facilement dans la plupart des espaces. Son coloris bois clair apporte une touche de luminosité et de douceur à votre chambre, créant une atmosphère apaisante. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Matelas 140x190 cm 8 HEURES FUTE : Confort et soutien optimal fabriqué en France</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Confort sur mesure pour des nuits paisibles
+Le matelas 140x190 cm 8 HEURES FUTE est un choix idéal pour ceux qui recherchent un confort équilibré et un soutien medium. Grâce à sa technologie de ressorts ensachés, ce matelas offre une indépendance de couchage remarquable, permettant de ne pas ressentir les mouvements de son partenaire. Fabriqué en France, il répond aux besoins des couples ou des personnes seules souhaitant un matelas deux places qui s'adapte parfaitement à leur morphologie. Son accueil ferme et son épaisseur de 21 cm garantissent un sommeil réparateur, quelle que soit la saison.
+Technologie avancée et fabrication française
+Ce matelas 8 HEURES FUTE se distingue par sa suspension de 480 ressorts ensachés, qui assure une excellente circulation de l'air et un soutien durable. Le tissu stretch 100 % polyester optimise la ventilation, évacuant l'humidité pour un confort optimal. Avec ses deux faces de couchage, il s'adapte aux variations saisonnières, offrant une face été avec un garnissage fin et respirant, et une face hiver plus enveloppante. Sa fabrication en France est un gage de qualité, garantissant un produit conforme aux normes les plus exigeantes.
+Un matelas pour tous les dormeurs
+Le matelas 140x190 cm 8 HEURES FUTE est conçu pour s'adresser à un large public. Que vous soyez un couple ou une personne seule, ce matelas deux places s'intègre parfaitement dans votre chambre. Son soutien medium et son accueil ferme conviennent à ceux qui recherchent un équilibre entre fermeté et moelleux. Avec un poids de 32 kg, il est à la fois robuste et facile à manipuler. Ce matelas est idéal pour ceux qui souhaitent investir dans un produit de qualité, fabriqué en France, qui assure des nuits paisibles et confortables.
+</t>
+    </r>
   </si>
   <si>
     <r>
@@ -658,50 +690,8 @@
 - Diamètre d’une roulette : 50 mm
 - Poids : 20,6 kg
 - Capacité de charge statique max. : 150 kg
-Livraison :
-- 1 x Fauteuil de bureau
-- 1 x Kit de montage
-- 1 x Mode d’emploi
-Précautions de SONGMICS :
-- Évitez toute exposition prolongée au soleil.
-- Évitez tout contact avec des objets pointus ou tranchants.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">surface PU résistante à l'usure </t>
-  </si>
-  <si>
-    <t>teintes chêne kronberg et waterford</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> tissu stretch 100 % polyester</t>
-  </si>
-  <si>
-    <t>Blanc</t>
-  </si>
-  <si>
-    <t>métal</t>
-  </si>
-  <si>
-    <t>noir avec un plateau et des crochets en bois</t>
-  </si>
-  <si>
-    <t>coloris naturel et noir</t>
-  </si>
-  <si>
-    <t>Bois et Métal</t>
-  </si>
-  <si>
-    <t>Table séjour +4 chaises</t>
-  </si>
-  <si>
-    <t>Lot de 2 Chevets</t>
-  </si>
-  <si>
-    <t>Armoire 3 portes battante</t>
-  </si>
-  <si>
-    <t>Lot de 2 meubles WC</t>
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1316,7 +1306,7 @@
         <v>31</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>9</v>
@@ -1365,10 +1355,10 @@
         <v>46</v>
       </c>
       <c r="S1" s="26" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="T1" s="26" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="241.5" x14ac:dyDescent="0.45">
@@ -1433,10 +1423,10 @@
         <v>47</v>
       </c>
       <c r="S2" s="27" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="T2" s="27" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="115.5" x14ac:dyDescent="0.45">
@@ -1501,13 +1491,13 @@
         <v>48</v>
       </c>
       <c r="S3" s="27" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="T3" s="27" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" ht="220.5" x14ac:dyDescent="0.45">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="210" x14ac:dyDescent="0.45">
       <c r="A4" s="7" t="s">
         <v>19</v>
       </c>
@@ -1566,13 +1556,13 @@
         <v>6</v>
       </c>
       <c r="R4" s="15" t="s">
-        <v>49</v>
+        <v>83</v>
       </c>
       <c r="S4" s="27" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="T4" s="27" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="262.5" x14ac:dyDescent="0.45">
@@ -1583,7 +1573,7 @@
         <v>33</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D5" s="9">
         <v>120</v>
@@ -1634,13 +1624,13 @@
         <v>7</v>
       </c>
       <c r="R5" s="15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="S5" s="27" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="T5" s="27" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="252" x14ac:dyDescent="0.45">
@@ -1702,13 +1692,13 @@
         <v>9</v>
       </c>
       <c r="R6" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="S6" s="27" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="T6" s="27" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="241.5" x14ac:dyDescent="0.45">
@@ -1770,16 +1760,16 @@
         <v>6</v>
       </c>
       <c r="R7" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S7" s="27" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="T7" s="27" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="409.5" x14ac:dyDescent="0.45">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" ht="388.5" x14ac:dyDescent="0.45">
       <c r="A8" s="7" t="s">
         <v>23</v>
       </c>
@@ -1838,16 +1828,16 @@
         <v>5</v>
       </c>
       <c r="R8" s="15" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="S8" s="27" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="T8" s="27" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" ht="189" x14ac:dyDescent="0.45">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" ht="178.5" x14ac:dyDescent="0.45">
       <c r="A9" s="7" t="s">
         <v>24</v>
       </c>
@@ -1906,13 +1896,13 @@
         <v>9</v>
       </c>
       <c r="R9" s="15" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="S9" s="27" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="T9" s="27" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="252" x14ac:dyDescent="0.45">
@@ -1923,7 +1913,7 @@
         <v>34</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D10" s="9">
         <v>35</v>
@@ -1974,16 +1964,16 @@
         <v>7</v>
       </c>
       <c r="R10" s="15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="S10" s="27" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="T10" s="27" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" ht="378" x14ac:dyDescent="0.45">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="252" x14ac:dyDescent="0.45">
       <c r="A11" s="7" t="s">
         <v>26</v>
       </c>
@@ -2042,13 +2032,13 @@
         <v>7</v>
       </c>
       <c r="R11" s="15" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="S11" s="27" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="T11" s="27" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="252" x14ac:dyDescent="0.45">
@@ -2110,16 +2100,16 @@
         <v>1</v>
       </c>
       <c r="R12" s="15" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="S12" s="27" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="T12" s="27" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" ht="241.5" x14ac:dyDescent="0.45">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" ht="231" x14ac:dyDescent="0.45">
       <c r="A13" s="7" t="s">
         <v>28</v>
       </c>
@@ -2127,7 +2117,7 @@
         <v>34</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D13" s="9">
         <v>52</v>
@@ -2178,13 +2168,13 @@
         <v>8</v>
       </c>
       <c r="R13" s="15" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="S13" s="27" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="T13" s="27" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="126" x14ac:dyDescent="0.45">
@@ -2246,13 +2236,13 @@
         <v>4</v>
       </c>
       <c r="R14" s="15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="S14" s="27" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="T14" s="27" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="241.5" x14ac:dyDescent="0.45">
@@ -2263,7 +2253,7 @@
         <v>36</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="G15" s="10"/>
       <c r="H15" s="10" t="s">
@@ -2302,13 +2292,13 @@
         <v>6</v>
       </c>
       <c r="R15" s="15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="S15" s="27" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="T15" s="27" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Modification Status certains meubles
</commit_message>
<xml_diff>
--- a/docs/Box GardeMeuble.xlsx
+++ b/docs/Box GardeMeuble.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acboi\Documents\Projets\vente-meubles\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A4CDDD-5798-4E19-9CE6-08A88EEB60CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4152A46-4BF6-4185-8EE3-052B0A26FA6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FD343005-4382-4935-A274-266D1E9B84BE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="89">
   <si>
     <t>Table salon</t>
   </si>
@@ -679,6 +679,9 @@
 Ce canapé 3 places se distingue par sa fonctionnalité convertible, transformant votre salon en un espace de couchage confortable en un clin d'œil. Grâce à son matelas d'une épaisseur de 12 cm en mousse polyuréthane, il offre un couchage régulier de qualité, garantissant un sommeil réparateur. La structure en pin et contreplaqué assure une robustesse et une durabilité exceptionnelles, tandis que la suspension à ressorts zig-zag et sangle offre un soutien optimal. Le revêtement en 100% polyester est non seulement agréable au toucher, mais également facile à entretenir, assurant ainsi une longévité accrue.
 Avec ses dimensions généreuses de largeur 198 cm, hauteur 89 cm et profondeur 99 cm, le canapé s'adapte parfaitement aux espaces de vie modernes. Son coloris gris, à la fois sobre et élégant, s'harmonise avec une multitude de styles de décoration. </t>
     </r>
+  </si>
+  <si>
+    <t>Vendu</t>
   </si>
 </sst>
 </file>
@@ -1809,7 +1812,7 @@
         <v>52</v>
       </c>
       <c r="P8" s="14" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="Q8" s="14">
         <v>5</v>
@@ -1877,7 +1880,7 @@
         <v>40</v>
       </c>
       <c r="P9" s="14" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="Q9" s="14">
         <v>9</v>
@@ -1945,7 +1948,7 @@
         <v>28</v>
       </c>
       <c r="P10" s="14" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="Q10" s="14">
         <v>7</v>
@@ -2013,7 +2016,7 @@
         <v>120</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="Q11" s="14">
         <v>7</v>

</xml_diff>

<commit_message>
modif status reservé à disponible
</commit_message>
<xml_diff>
--- a/docs/Box GardeMeuble.xlsx
+++ b/docs/Box GardeMeuble.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acboi\Documents\Projets\vente-meubles\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A6C5F3-FCDA-4FF9-8644-4C131B70DAA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F15A99-4222-4FE4-806E-466C5114043E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FD343005-4382-4935-A274-266D1E9B84BE}"/>
   </bookViews>
@@ -1880,7 +1880,7 @@
         <v>40</v>
       </c>
       <c r="P9" s="14" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="Q9" s="14">
         <v>9</v>
@@ -1948,7 +1948,7 @@
         <v>28</v>
       </c>
       <c r="P10" s="14" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="Q10" s="14">
         <v>7</v>
@@ -2016,7 +2016,7 @@
         <v>120</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="Q11" s="14">
         <v>7</v>

</xml_diff>